<commit_message>
Add Tray Entry form sheet with SubmitTrayReturn macro
- New "Tray Entry" sheet: vertical form with Route, Area, Tray Count,
  Date Returned, Inspector fields (same mobile-friendly layout)
- VBA SubmitTrayReturn macro: validates, appends to Tray Returns, clears form
- Now 3 macros in VBA Code sheet: SubmitProductReturn, SubmitTrayReturn,
  GenerateSensoryReport

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/QAReturns.xlsx
+++ b/output/QAReturns.xlsx
@@ -6,18 +6,19 @@
   <sheets>
     <sheet sheetId="1" name="Lookups" state="veryHidden" r:id="rId4"/>
     <sheet sheetId="2" name="Data Entry" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Product Returns" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Tray Returns" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Summary" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Report Generator" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="VBA Code" state="visible" r:id="rId10"/>
+    <sheet sheetId="3" name="Tray Entry" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Product Returns" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Tray Returns" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Summary" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Report Generator" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="VBA Code" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="459">
   <si>
     <t>Routes</t>
   </si>
@@ -298,6 +299,15 @@
     <t/>
   </si>
   <si>
+    <t>Tray Returns Entry</t>
+  </si>
+  <si>
+    <t>Tray Count</t>
+  </si>
+  <si>
+    <t>Run macro "SubmitTrayReturn" to add this entry (Alt+F8)</t>
+  </si>
+  <si>
     <t>Record #</t>
   </si>
   <si>
@@ -331,9 +341,6 @@
     <t>Area overstocked. All units in sellable condition.</t>
   </si>
   <si>
-    <t>Tray Count</t>
-  </si>
-  <si>
     <t>QA Returns Summary</t>
   </si>
   <si>
@@ -406,13 +413,16 @@
     <t>' QA Returns — VBA Macros</t>
   </si>
   <si>
-    <t>' Contains two macros:</t>
+    <t>' Contains three macros:</t>
   </si>
   <si>
     <t>'   1) SubmitProductReturn  — adds Data Entry form to Product Returns</t>
   </si>
   <si>
-    <t>'   2) GenerateSensoryReport — generates Sensory Evaluation report</t>
+    <t>'   2) SubmitTrayReturn     — adds Tray Entry form to Tray Returns</t>
+  </si>
+  <si>
+    <t>'   3) GenerateSensoryReport — generates Sensory Evaluation report</t>
   </si>
   <si>
     <t>Sub SubmitProductReturn()</t>
@@ -679,6 +689,66 @@
     <t>End Sub</t>
   </si>
   <si>
+    <t>Sub SubmitTrayReturn()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dim wsTR As Worksheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Set wsForm = ThisWorkbook.Sheets("Tray Entry")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Set wsTR = ThisWorkbook.Sheets("Tray Returns")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dim fTrayCount As Variant:  fTrayCount = wsForm.Range("B6").Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dim fReturned As Variant:   fReturned = wsForm.Range("B7").Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dim fInspector As String:   fInspector = Trim(CStr(wsForm.Range("B8").Value))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    If Not IsNumeric(fTrayCount) Or CLng(fTrayCount) &lt; 0 Then</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        MsgBox "Tray Count must be a number &gt;= 0.", vbExclamation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ' ── Find next empty row in Tray Returns (check col C = Route) ──</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        If wsTR.Cells(i, 3).Value &lt;&gt; "" Then</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        MsgBox "Tray Returns sheet is full (500 rows).", vbExclamation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ' ── Write data to Tray Returns ──</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsTR.Cells(nextRow, 3).Value = fRoute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsTR.Cells(nextRow, 4).Value = fArea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsTR.Cells(nextRow, 5).Value = CLng(fTrayCount)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    If IsDate(fReturned) Then wsTR.Cells(nextRow, 6).Value = CDate(fReturned)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsTR.Cells(nextRow, 7).Value = fInspector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsForm.Range("A12").Value = "Record #" &amp; (nextRow - 1) &amp; " added successfully!"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    MsgBox "Tray record added as row " &amp; nextRow &amp; " in Tray Returns!", vbInformation</t>
+  </si>
+  <si>
     <t>Sub GenerateSensoryReport()</t>
   </si>
   <si>
@@ -688,16 +758,10 @@
     <t xml:space="preserve">    Dim wsGen As Worksheet</t>
   </si>
   <si>
-    <t xml:space="preserve">    Dim wsTR As Worksheet</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Dim wsOut As Worksheet</t>
   </si>
   <si>
     <t xml:space="preserve">    Set wsGen = ThisWorkbook.Sheets("Report Generator")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Set wsTR = ThisWorkbook.Sheets("Tray Returns")</t>
   </si>
   <si>
     <t xml:space="preserve">    ' ── Read inputs ──</t>
@@ -2316,6 +2380,96 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="4"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="4"/>
+    </row>
+    <row r="9" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="6"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A12:B12"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid" error="Please enter a valid Route." sqref="B4">
+      <formula1>Routes</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid" error="Please enter a valid Area." sqref="B5">
+      <formula1>INDIRECT("Route_"&amp;SUBSTITUTE(B4," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid" error="Please enter a valid Tray Count." sqref="B6">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid" error="Please enter a valid Inspector." sqref="B8">
+      <formula1>Users</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O501"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2334,10 +2488,10 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>78</v>
@@ -2402,7 +2556,7 @@
         <v>5</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I2" s="10">
         <v>46072.66666666667</v>
@@ -2420,7 +2574,7 @@
         <v>92</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="O2" s="11" t="s">
         <v>14</v>
@@ -2449,7 +2603,7 @@
         <v>12</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I3" s="13">
         <v>46074.66666666667</v>
@@ -2467,7 +2621,7 @@
         <v>92</v>
       </c>
       <c r="N3" s="14" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="O3" s="14" t="s">
         <v>25</v>
@@ -2514,7 +2668,7 @@
         <v>92</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O4" s="11" t="s">
         <v>14</v>
@@ -2543,7 +2697,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I5" s="13">
         <v>46076.66666666667</v>
@@ -2561,7 +2715,7 @@
         <v>92</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="O5" s="14" t="s">
         <v>25</v>
@@ -2590,7 +2744,7 @@
         <v>6</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="I6" s="10">
         <v>46073.66666666667</v>
@@ -2608,7 +2762,7 @@
         <v>92</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="O6" s="11" t="s">
         <v>14</v>
@@ -16052,7 +16206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G501"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -16067,10 +16221,10 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>78</v>
@@ -16079,7 +16233,7 @@
         <v>79</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>86</v>
@@ -24114,7 +24268,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -24125,7 +24279,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -24133,12 +24287,12 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B4" s="18">
         <f>COUNTA('Product Returns'!C2:C501)-COUNTBLANK('Product Returns'!C2:C501)</f>
@@ -24146,7 +24300,7 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B5" s="18">
         <f>SUMPRODUCT(('Product Returns'!G2:G501&lt;&gt;"")*1*('Product Returns'!G2:G501))</f>
@@ -24154,7 +24308,7 @@
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" s="18">
         <f>COUNTIF('Product Returns'!L2:L501,"&lt;&gt;"&amp;"")-COUNTIF('Product Returns'!L2:L501,"Good Condition")</f>
@@ -24162,7 +24316,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -24170,7 +24324,7 @@
         <v>78</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>82</v>
@@ -24233,7 +24387,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -24241,7 +24395,7 @@
         <v>87</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -24317,7 +24471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -24329,14 +24483,14 @@
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>11</v>
@@ -24344,15 +24498,15 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B5" s="24">
-        <v>46083.13418952546</v>
+        <v>46083.13896923611</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B6" s="25">
         <v>0</v>
@@ -24360,15 +24514,15 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B8" s="24">
-        <v>46083.13418952546</v>
+        <v>46083.13896923611</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B9" s="25">
         <v>0.9999</v>
@@ -24376,47 +24530,47 @@
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="28" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B16" s="28"/>
       <c r="C16" s="28"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="28" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B17" s="28"/>
       <c r="C17" s="28"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="28" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28"/>
@@ -24441,9 +24595,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A465"/>
+  <dimension ref="A1:A541"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="130" customWidth="1"/>
@@ -24451,647 +24605,647 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
-        <v>132</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="30" t="s">
-        <v>92</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="30" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="30" t="s">
-        <v>137</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="30" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="30" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="30" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="30" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="30" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="30" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="30" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="30" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="30" t="s">
-        <v>92</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="30" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="30" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="30" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="30" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="30" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="30" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="30" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="30" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="30" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="30" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="30" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="30" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="30" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="30" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="30" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="30" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="30" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="30" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="30" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="30" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="30" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="30" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="30" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="30" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="30" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="30" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="30" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="30" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="30" t="s">
-        <v>92</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="30" t="s">
-        <v>184</v>
+        <v>92</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="30" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="30" t="s">
-        <v>155</v>
+        <v>188</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="30" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="30" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="30" t="s">
-        <v>186</v>
+        <v>92</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="30" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="30" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="30" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="30" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="30" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="30" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="30" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="30" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="30" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="30" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="30" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="30" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="30" t="s">
-        <v>92</v>
+        <v>203</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="30" t="s">
-        <v>201</v>
+        <v>92</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="30" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="30" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="30" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="30" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="30" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="30" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="30" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="30" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="30" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="30" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="30" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="30" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="30" t="s">
-        <v>92</v>
+        <v>217</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="30" t="s">
-        <v>215</v>
+        <v>92</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="30" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="30" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="30" t="s">
-        <v>92</v>
+        <v>220</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="30" t="s">
-        <v>218</v>
+        <v>92</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="30" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="30" t="s">
-        <v>92</v>
+        <v>222</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="30" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="30" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="30" t="s">
-        <v>220</v>
+        <v>92</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="30" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="30" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="30" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="30" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="30" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="30" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
@@ -25101,142 +25255,142 @@
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="30" t="s">
-        <v>225</v>
+        <v>140</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="30" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="30" t="s">
-        <v>226</v>
+        <v>142</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" s="30" t="s">
-        <v>92</v>
+        <v>227</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" s="30" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" s="30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="30" t="s">
-        <v>229</v>
+        <v>92</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" s="30" t="s">
-        <v>230</v>
+        <v>154</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" s="30" t="s">
-        <v>231</v>
+        <v>155</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" s="30" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" s="30" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" s="30" t="s">
-        <v>232</v>
+        <v>159</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" s="30" t="s">
-        <v>233</v>
+        <v>160</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="30" t="s">
-        <v>234</v>
+        <v>161</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="30" t="s">
-        <v>235</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" s="30" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" s="30" t="s">
-        <v>236</v>
+        <v>159</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="30" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" s="30" t="s">
-        <v>155</v>
+        <v>231</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="30" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" s="30" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="30" t="s">
-        <v>238</v>
+        <v>159</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" s="30" t="s">
-        <v>239</v>
+        <v>175</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" s="30" t="s">
-        <v>240</v>
+        <v>176</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" s="30" t="s">
-        <v>241</v>
+        <v>171</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="30" t="s">
-        <v>242</v>
+        <v>158</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="30" t="s">
-        <v>243</v>
+        <v>159</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
@@ -25246,207 +25400,207 @@
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" s="30" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="30" t="s">
-        <v>245</v>
+        <v>179</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" s="30" t="s">
-        <v>92</v>
+        <v>180</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="30" t="s">
-        <v>246</v>
+        <v>181</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" s="30" t="s">
-        <v>247</v>
+        <v>182</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" s="30" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" s="30" t="s">
-        <v>249</v>
+        <v>184</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" s="30" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" s="30" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" s="30" t="s">
-        <v>250</v>
+        <v>92</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" s="30" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" s="30" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" s="30" t="s">
-        <v>179</v>
+        <v>158</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" s="30" t="s">
-        <v>252</v>
+        <v>159</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" s="30" t="s">
-        <v>183</v>
+        <v>92</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" s="30" t="s">
-        <v>92</v>
+        <v>235</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" s="30" t="s">
-        <v>253</v>
+        <v>190</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" s="30" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" s="30" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" s="30" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" s="30" t="s">
-        <v>92</v>
+        <v>239</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" s="30" t="s">
-        <v>257</v>
+        <v>240</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" s="30" t="s">
-        <v>258</v>
+        <v>92</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184" s="30" t="s">
-        <v>259</v>
+        <v>204</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A185" s="30" t="s">
-        <v>260</v>
+        <v>205</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A186" s="30" t="s">
-        <v>261</v>
+        <v>206</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" s="30" t="s">
-        <v>262</v>
+        <v>207</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" s="30" t="s">
-        <v>263</v>
+        <v>208</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" s="30" t="s">
-        <v>264</v>
+        <v>209</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" s="30" t="s">
-        <v>265</v>
+        <v>92</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" s="30" t="s">
-        <v>182</v>
+        <v>218</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" s="30" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" s="30" t="s">
-        <v>92</v>
+        <v>220</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" s="30" t="s">
-        <v>266</v>
+        <v>92</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="30" t="s">
-        <v>267</v>
+        <v>242</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" s="30" t="s">
-        <v>268</v>
+        <v>222</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="30" t="s">
-        <v>269</v>
+        <v>92</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A198" s="30" t="s">
-        <v>270</v>
+        <v>129</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" s="30" t="s">
-        <v>271</v>
+        <v>92</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" s="30" t="s">
-        <v>155</v>
+        <v>243</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" s="30" t="s">
-        <v>156</v>
+        <v>244</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.25">
@@ -25456,247 +25610,247 @@
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" s="30" t="s">
-        <v>272</v>
+        <v>245</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" s="30" t="s">
-        <v>273</v>
+        <v>137</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" s="30" t="s">
-        <v>274</v>
+        <v>224</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" s="30" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" s="30" t="s">
-        <v>258</v>
+        <v>92</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" s="30" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A209" s="30" t="s">
-        <v>261</v>
+        <v>139</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A210" s="30" t="s">
-        <v>262</v>
+        <v>226</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A211" s="30" t="s">
-        <v>275</v>
+        <v>92</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A212" s="30" t="s">
-        <v>276</v>
+        <v>248</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A213" s="30" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A214" s="30" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A215" s="30" t="s">
-        <v>182</v>
+        <v>251</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A216" s="30" t="s">
-        <v>183</v>
+        <v>252</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A217" s="30" t="s">
-        <v>92</v>
+        <v>158</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A218" s="30" t="s">
-        <v>277</v>
+        <v>159</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A219" s="30" t="s">
-        <v>278</v>
+        <v>92</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A220" s="30" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A221" s="30" t="s">
-        <v>280</v>
+        <v>254</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A222" s="30" t="s">
-        <v>281</v>
+        <v>255</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A223" s="30" t="s">
-        <v>282</v>
+        <v>256</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A224" s="30" t="s">
-        <v>283</v>
+        <v>92</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A225" s="30" t="s">
-        <v>284</v>
+        <v>257</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A226" s="30" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A227" s="30" t="s">
-        <v>286</v>
+        <v>158</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A228" s="30" t="s">
-        <v>287</v>
+        <v>159</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A229" s="30" t="s">
-        <v>288</v>
+        <v>92</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A230" s="30" t="s">
-        <v>289</v>
+        <v>259</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A231" s="30" t="s">
-        <v>290</v>
+        <v>260</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A232" s="30" t="s">
-        <v>291</v>
+        <v>261</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A233" s="30" t="s">
-        <v>292</v>
+        <v>262</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A234" s="30" t="s">
-        <v>293</v>
+        <v>263</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A235" s="30" t="s">
-        <v>294</v>
+        <v>264</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A236" s="30" t="s">
-        <v>295</v>
+        <v>92</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A237" s="30" t="s">
-        <v>296</v>
+        <v>265</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A238" s="30" t="s">
-        <v>297</v>
+        <v>266</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A239" s="30" t="s">
-        <v>264</v>
+        <v>92</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A240" s="30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A241" s="30" t="s">
-        <v>182</v>
+        <v>268</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A242" s="30" t="s">
-        <v>183</v>
+        <v>269</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A243" s="30" t="s">
-        <v>92</v>
+        <v>270</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A244" s="30" t="s">
-        <v>298</v>
+        <v>181</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A245" s="30" t="s">
-        <v>299</v>
+        <v>182</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A246" s="30" t="s">
-        <v>300</v>
+        <v>271</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A247" s="30" t="s">
-        <v>301</v>
+        <v>186</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A248" s="30" t="s">
-        <v>302</v>
+        <v>272</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A249" s="30" t="s">
-        <v>303</v>
+        <v>182</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A250" s="30" t="s">
-        <v>304</v>
+        <v>273</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A251" s="30" t="s">
-        <v>305</v>
+        <v>186</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.25">
@@ -25706,127 +25860,127 @@
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A253" s="30" t="s">
-        <v>306</v>
+        <v>274</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A254" s="30" t="s">
-        <v>307</v>
+        <v>275</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A255" s="30" t="s">
-        <v>308</v>
+        <v>276</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A256" s="30" t="s">
-        <v>309</v>
+        <v>277</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A257" s="30" t="s">
-        <v>310</v>
+        <v>92</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A258" s="30" t="s">
-        <v>311</v>
+        <v>278</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A259" s="30" t="s">
-        <v>312</v>
+        <v>279</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A260" s="30" t="s">
-        <v>313</v>
+        <v>280</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A261" s="30" t="s">
-        <v>314</v>
+        <v>281</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A262" s="30" t="s">
-        <v>315</v>
+        <v>282</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A263" s="30" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A264" s="30" t="s">
-        <v>316</v>
+        <v>284</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A265" s="30" t="s">
-        <v>183</v>
+        <v>285</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A266" s="30" t="s">
-        <v>92</v>
+        <v>286</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A267" s="30" t="s">
-        <v>317</v>
+        <v>185</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A268" s="30" t="s">
-        <v>318</v>
+        <v>186</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A269" s="30" t="s">
-        <v>319</v>
+        <v>92</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A270" s="30" t="s">
-        <v>320</v>
+        <v>287</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A271" s="30" t="s">
-        <v>321</v>
+        <v>288</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A272" s="30" t="s">
-        <v>322</v>
+        <v>289</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A273" s="30" t="s">
-        <v>323</v>
+        <v>290</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A274" s="30" t="s">
-        <v>324</v>
+        <v>291</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A275" s="30" t="s">
-        <v>92</v>
+        <v>292</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A276" s="30" t="s">
-        <v>325</v>
+        <v>158</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A277" s="30" t="s">
-        <v>326</v>
+        <v>159</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.25">
@@ -25836,522 +25990,522 @@
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A279" s="30" t="s">
-        <v>327</v>
+        <v>293</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A280" s="30" t="s">
-        <v>328</v>
+        <v>294</v>
       </c>
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A281" s="30" t="s">
-        <v>329</v>
+        <v>295</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A282" s="30" t="s">
-        <v>330</v>
+        <v>278</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A283" s="30" t="s">
-        <v>331</v>
+        <v>279</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A284" s="30" t="s">
-        <v>92</v>
+        <v>281</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A285" s="30" t="s">
-        <v>332</v>
+        <v>282</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A286" s="30" t="s">
-        <v>333</v>
+        <v>283</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A287" s="30" t="s">
-        <v>334</v>
+        <v>296</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A288" s="30" t="s">
-        <v>335</v>
+        <v>297</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A289" s="30" t="s">
-        <v>336</v>
+        <v>285</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A290" s="30" t="s">
-        <v>92</v>
+        <v>286</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A291" s="30" t="s">
-        <v>337</v>
+        <v>185</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A292" s="30" t="s">
-        <v>333</v>
+        <v>186</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A293" s="30" t="s">
-        <v>334</v>
+        <v>92</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A294" s="30" t="s">
-        <v>335</v>
+        <v>298</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A295" s="30" t="s">
-        <v>336</v>
+        <v>299</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A296" s="30" t="s">
-        <v>92</v>
+        <v>300</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A297" s="30" t="s">
-        <v>338</v>
+        <v>301</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A298" s="30" t="s">
-        <v>339</v>
+        <v>302</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A299" s="30" t="s">
-        <v>340</v>
+        <v>303</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A300" s="30" t="s">
-        <v>341</v>
+        <v>304</v>
       </c>
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A301" s="30" t="s">
-        <v>342</v>
+        <v>305</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A302" s="30" t="s">
-        <v>343</v>
+        <v>306</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A303" s="30" t="s">
-        <v>92</v>
+        <v>307</v>
       </c>
     </row>
     <row r="304" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A304" s="30" t="s">
-        <v>344</v>
+        <v>308</v>
       </c>
     </row>
     <row r="305" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A305" s="30" t="s">
-        <v>345</v>
+        <v>309</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A306" s="30" t="s">
-        <v>346</v>
+        <v>310</v>
       </c>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A307" s="30" t="s">
-        <v>347</v>
+        <v>311</v>
       </c>
     </row>
     <row r="308" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A308" s="30" t="s">
-        <v>348</v>
+        <v>312</v>
       </c>
     </row>
     <row r="309" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A309" s="30" t="s">
-        <v>92</v>
+        <v>313</v>
       </c>
     </row>
     <row r="310" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A310" s="30" t="s">
-        <v>349</v>
+        <v>314</v>
       </c>
     </row>
     <row r="311" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A311" s="30" t="s">
-        <v>350</v>
+        <v>315</v>
       </c>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A312" s="30" t="s">
-        <v>351</v>
+        <v>316</v>
       </c>
     </row>
     <row r="313" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A313" s="30" t="s">
-        <v>92</v>
+        <v>317</v>
       </c>
     </row>
     <row r="314" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A314" s="30" t="s">
-        <v>352</v>
+        <v>318</v>
       </c>
     </row>
     <row r="315" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A315" s="30" t="s">
-        <v>353</v>
+        <v>285</v>
       </c>
     </row>
     <row r="316" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A316" s="30" t="s">
-        <v>182</v>
+        <v>286</v>
       </c>
     </row>
     <row r="317" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A317" s="30" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="318" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A318" s="30" t="s">
-        <v>354</v>
+        <v>186</v>
       </c>
     </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A319" s="30" t="s">
-        <v>355</v>
+        <v>92</v>
       </c>
     </row>
     <row r="320" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A320" s="30" t="s">
-        <v>356</v>
+        <v>319</v>
       </c>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A321" s="30" t="s">
-        <v>357</v>
+        <v>320</v>
       </c>
     </row>
     <row r="322" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A322" s="30" t="s">
-        <v>358</v>
+        <v>321</v>
       </c>
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A323" s="30" t="s">
-        <v>359</v>
+        <v>322</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A324" s="30" t="s">
-        <v>92</v>
+        <v>323</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A325" s="30" t="s">
-        <v>360</v>
+        <v>324</v>
       </c>
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A326" s="30" t="s">
-        <v>361</v>
+        <v>325</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A327" s="30" t="s">
-        <v>362</v>
+        <v>326</v>
       </c>
     </row>
     <row r="328" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A328" s="30" t="s">
-        <v>363</v>
+        <v>92</v>
       </c>
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A329" s="30" t="s">
-        <v>364</v>
+        <v>327</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A330" s="30" t="s">
-        <v>365</v>
+        <v>328</v>
       </c>
     </row>
     <row r="331" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A331" s="30" t="s">
-        <v>366</v>
+        <v>329</v>
       </c>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A332" s="30" t="s">
-        <v>367</v>
+        <v>330</v>
       </c>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A333" s="30" t="s">
-        <v>265</v>
+        <v>331</v>
       </c>
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A334" s="30" t="s">
-        <v>368</v>
+        <v>332</v>
       </c>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A335" s="30" t="s">
-        <v>369</v>
+        <v>333</v>
       </c>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A336" s="30" t="s">
-        <v>370</v>
+        <v>334</v>
       </c>
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A337" s="30" t="s">
-        <v>371</v>
+        <v>335</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A338" s="30" t="s">
-        <v>372</v>
+        <v>336</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A339" s="30" t="s">
-        <v>373</v>
+        <v>286</v>
       </c>
     </row>
     <row r="340" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A340" s="30" t="s">
-        <v>374</v>
+        <v>337</v>
       </c>
     </row>
     <row r="341" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A341" s="30" t="s">
-        <v>375</v>
+        <v>186</v>
       </c>
     </row>
     <row r="342" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A342" s="30" t="s">
-        <v>376</v>
+        <v>92</v>
       </c>
     </row>
     <row r="343" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A343" s="30" t="s">
-        <v>297</v>
+        <v>338</v>
       </c>
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A344" s="30" t="s">
-        <v>264</v>
+        <v>339</v>
       </c>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A345" s="30" t="s">
-        <v>265</v>
+        <v>340</v>
       </c>
     </row>
     <row r="346" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A346" s="30" t="s">
-        <v>377</v>
+        <v>341</v>
       </c>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A347" s="30" t="s">
-        <v>92</v>
+        <v>342</v>
       </c>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A348" s="30" t="s">
-        <v>378</v>
+        <v>343</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A349" s="30" t="s">
-        <v>379</v>
+        <v>344</v>
       </c>
     </row>
     <row r="350" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A350" s="30" t="s">
-        <v>380</v>
+        <v>345</v>
       </c>
     </row>
     <row r="351" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A351" s="30" t="s">
-        <v>381</v>
+        <v>92</v>
       </c>
     </row>
     <row r="352" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A352" s="30" t="s">
-        <v>382</v>
+        <v>346</v>
       </c>
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A353" s="30" t="s">
-        <v>383</v>
+        <v>347</v>
       </c>
     </row>
     <row r="354" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A354" s="30" t="s">
-        <v>384</v>
+        <v>92</v>
       </c>
     </row>
     <row r="355" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A355" s="30" t="s">
-        <v>92</v>
+        <v>348</v>
       </c>
     </row>
     <row r="356" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A356" s="30" t="s">
-        <v>385</v>
+        <v>349</v>
       </c>
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A357" s="30" t="s">
-        <v>386</v>
+        <v>350</v>
       </c>
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A358" s="30" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A359" s="30" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A360" s="30" t="s">
-        <v>359</v>
+        <v>92</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A361" s="30" t="s">
-        <v>92</v>
+        <v>353</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A362" s="30" t="s">
-        <v>387</v>
+        <v>354</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A363" s="30" t="s">
-        <v>388</v>
+        <v>355</v>
       </c>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A364" s="30" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A365" s="30" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
     </row>
     <row r="366" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A366" s="30" t="s">
-        <v>389</v>
+        <v>92</v>
       </c>
     </row>
     <row r="367" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A367" s="30" t="s">
-        <v>265</v>
+        <v>358</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A368" s="30" t="s">
-        <v>368</v>
+        <v>354</v>
       </c>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A369" s="30" t="s">
-        <v>92</v>
+        <v>355</v>
       </c>
     </row>
     <row r="370" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A370" s="30" t="s">
-        <v>390</v>
+        <v>356</v>
       </c>
     </row>
     <row r="371" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A371" s="30" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A372" s="30" t="s">
-        <v>386</v>
+        <v>92</v>
       </c>
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A373" s="30" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A374" s="30" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="375" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A375" s="30" t="s">
-        <v>391</v>
+        <v>361</v>
       </c>
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A376" s="30" t="s">
-        <v>92</v>
+        <v>362</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A377" s="30" t="s">
-        <v>392</v>
+        <v>363</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A378" s="30" t="s">
-        <v>393</v>
+        <v>364</v>
       </c>
     </row>
     <row r="379" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A379" s="30" t="s">
-        <v>394</v>
+        <v>92</v>
       </c>
     </row>
     <row r="380" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A380" s="30" t="s">
-        <v>395</v>
+        <v>365</v>
       </c>
     </row>
     <row r="381" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A381" s="30" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A382" s="30" t="s">
-        <v>396</v>
+        <v>367</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.25">
@@ -26361,382 +26515,382 @@
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A384" s="30" t="s">
-        <v>92</v>
+        <v>369</v>
       </c>
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A385" s="30" t="s">
-        <v>397</v>
+        <v>92</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A386" s="30" t="s">
-        <v>398</v>
+        <v>370</v>
       </c>
     </row>
     <row r="387" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A387" s="30" t="s">
-        <v>399</v>
+        <v>371</v>
       </c>
     </row>
     <row r="388" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A388" s="30" t="s">
-        <v>400</v>
+        <v>372</v>
       </c>
     </row>
     <row r="389" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A389" s="30" t="s">
-        <v>401</v>
+        <v>92</v>
       </c>
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A390" s="30" t="s">
-        <v>402</v>
+        <v>373</v>
       </c>
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A391" s="30" t="s">
-        <v>403</v>
+        <v>374</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A392" s="30" t="s">
-        <v>404</v>
+        <v>185</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A393" s="30" t="s">
-        <v>264</v>
+        <v>92</v>
       </c>
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A394" s="30" t="s">
-        <v>405</v>
+        <v>375</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A395" s="30" t="s">
-        <v>92</v>
+        <v>376</v>
       </c>
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A396" s="30" t="s">
-        <v>406</v>
+        <v>377</v>
       </c>
     </row>
     <row r="397" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A397" s="30" t="s">
-        <v>407</v>
+        <v>378</v>
       </c>
     </row>
     <row r="398" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A398" s="30" t="s">
-        <v>408</v>
+        <v>379</v>
       </c>
     </row>
     <row r="399" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A399" s="30" t="s">
-        <v>409</v>
+        <v>380</v>
       </c>
     </row>
     <row r="400" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A400" s="30" t="s">
-        <v>410</v>
+        <v>92</v>
       </c>
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A401" s="30" t="s">
-        <v>411</v>
+        <v>381</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A402" s="30" t="s">
-        <v>412</v>
+        <v>382</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A403" s="30" t="s">
-        <v>297</v>
+        <v>383</v>
       </c>
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A404" s="30" t="s">
-        <v>413</v>
+        <v>384</v>
       </c>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A405" s="30" t="s">
-        <v>414</v>
+        <v>385</v>
       </c>
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A406" s="30" t="s">
-        <v>92</v>
+        <v>386</v>
       </c>
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A407" s="30" t="s">
-        <v>415</v>
+        <v>387</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A408" s="30" t="s">
-        <v>416</v>
+        <v>388</v>
       </c>
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A409" s="30" t="s">
-        <v>417</v>
+        <v>286</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A410" s="30" t="s">
-        <v>92</v>
+        <v>389</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A411" s="30" t="s">
-        <v>418</v>
+        <v>390</v>
       </c>
     </row>
     <row r="412" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A412" s="30" t="s">
-        <v>419</v>
+        <v>391</v>
       </c>
     </row>
     <row r="413" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A413" s="30" t="s">
-        <v>420</v>
+        <v>392</v>
       </c>
     </row>
     <row r="414" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A414" s="30" t="s">
-        <v>421</v>
+        <v>393</v>
       </c>
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A415" s="30" t="s">
-        <v>422</v>
+        <v>394</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A416" s="30" t="s">
-        <v>92</v>
+        <v>395</v>
       </c>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A417" s="30" t="s">
-        <v>423</v>
+        <v>396</v>
       </c>
     </row>
     <row r="418" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A418" s="30" t="s">
-        <v>419</v>
+        <v>397</v>
       </c>
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A419" s="30" t="s">
-        <v>420</v>
+        <v>318</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A420" s="30" t="s">
-        <v>421</v>
+        <v>285</v>
       </c>
     </row>
     <row r="421" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A421" s="30" t="s">
-        <v>422</v>
+        <v>286</v>
       </c>
     </row>
     <row r="422" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A422" s="30" t="s">
-        <v>92</v>
+        <v>398</v>
       </c>
     </row>
     <row r="423" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A423" s="30" t="s">
-        <v>424</v>
+        <v>92</v>
       </c>
     </row>
     <row r="424" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A424" s="30" t="s">
-        <v>419</v>
+        <v>399</v>
       </c>
     </row>
     <row r="425" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A425" s="30" t="s">
-        <v>420</v>
+        <v>400</v>
       </c>
     </row>
     <row r="426" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A426" s="30" t="s">
-        <v>421</v>
+        <v>401</v>
       </c>
     </row>
     <row r="427" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A427" s="30" t="s">
-        <v>422</v>
+        <v>402</v>
       </c>
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A428" s="30" t="s">
-        <v>92</v>
+        <v>403</v>
       </c>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A429" s="30" t="s">
-        <v>425</v>
+        <v>404</v>
       </c>
     </row>
     <row r="430" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A430" s="30" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A431" s="30" t="s">
-        <v>420</v>
+        <v>92</v>
       </c>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A432" s="30" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A433" s="30" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
     </row>
     <row r="434" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A434" s="30" t="s">
-        <v>92</v>
+        <v>379</v>
       </c>
     </row>
     <row r="435" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A435" s="30" t="s">
-        <v>426</v>
+        <v>378</v>
       </c>
     </row>
     <row r="436" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A436" s="30" t="s">
-        <v>427</v>
+        <v>380</v>
       </c>
     </row>
     <row r="437" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A437" s="30" t="s">
-        <v>428</v>
+        <v>92</v>
       </c>
     </row>
     <row r="438" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A438" s="30" t="s">
-        <v>429</v>
+        <v>408</v>
       </c>
     </row>
     <row r="439" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A439" s="30" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A440" s="30" t="s">
-        <v>420</v>
+        <v>384</v>
       </c>
     </row>
     <row r="441" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A441" s="30" t="s">
-        <v>421</v>
+        <v>385</v>
       </c>
     </row>
     <row r="442" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A442" s="30" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A443" s="30" t="s">
-        <v>92</v>
+        <v>286</v>
       </c>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A444" s="30" t="s">
-        <v>430</v>
+        <v>389</v>
       </c>
     </row>
     <row r="445" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A445" s="30" t="s">
-        <v>419</v>
+        <v>92</v>
       </c>
     </row>
     <row r="446" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A446" s="30" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="447" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A447" s="30" t="s">
-        <v>421</v>
+        <v>376</v>
       </c>
     </row>
     <row r="448" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A448" s="30" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
     </row>
     <row r="449" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A449" s="30" t="s">
-        <v>92</v>
+        <v>379</v>
       </c>
     </row>
     <row r="450" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A450" s="30" t="s">
-        <v>431</v>
+        <v>378</v>
       </c>
     </row>
     <row r="451" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A451" s="30" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
     </row>
     <row r="452" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A452" s="30" t="s">
-        <v>420</v>
+        <v>92</v>
       </c>
     </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A453" s="30" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
     </row>
     <row r="454" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A454" s="30" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
     </row>
     <row r="455" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A455" s="30" t="s">
-        <v>92</v>
+        <v>415</v>
       </c>
     </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A456" s="30" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A457" s="30" t="s">
-        <v>432</v>
+        <v>384</v>
       </c>
     </row>
     <row r="458" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A458" s="30" t="s">
-        <v>182</v>
+        <v>417</v>
       </c>
     </row>
     <row r="459" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A459" s="30" t="s">
-        <v>433</v>
+        <v>389</v>
       </c>
     </row>
     <row r="460" spans="1:1" x14ac:dyDescent="0.25">
@@ -26746,27 +26900,407 @@
     </row>
     <row r="461" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A461" s="30" t="s">
-        <v>434</v>
+        <v>418</v>
       </c>
     </row>
     <row r="462" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A462" s="30" t="s">
-        <v>435</v>
+        <v>419</v>
       </c>
     </row>
     <row r="463" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A463" s="30" t="s">
-        <v>436</v>
+        <v>420</v>
       </c>
     </row>
     <row r="464" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A464" s="30" t="s">
-        <v>437</v>
+        <v>421</v>
       </c>
     </row>
     <row r="465" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A465" s="30" t="s">
-        <v>219</v>
+        <v>422</v>
+      </c>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A466" s="30" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A467" s="30" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="468" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A468" s="30" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="469" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A469" s="30" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A470" s="30" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="471" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A471" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="472" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A472" s="30" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="473" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A473" s="30" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="474" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A474" s="30" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="475" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A475" s="30" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="476" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A476" s="30" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="477" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A477" s="30" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="478" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A478" s="30" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="479" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A479" s="30" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="480" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A480" s="30" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="481" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A481" s="30" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="482" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A482" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="483" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A483" s="30" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="484" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A484" s="30" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="485" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A485" s="30" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="486" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A486" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="487" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A487" s="30" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="488" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A488" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="489" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A489" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="490" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A490" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="491" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A491" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="492" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A492" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="493" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A493" s="30" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="494" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A494" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="495" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A495" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="496" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A496" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="497" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A497" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="498" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A498" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="499" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A499" s="30" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="500" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A500" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="501" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A501" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="502" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A502" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="503" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A503" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="504" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A504" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="505" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A505" s="30" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A506" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="507" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A507" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="508" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A508" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="509" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A509" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="510" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A510" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="511" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A511" s="30" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="512" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A512" s="30" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="513" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A513" s="30" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="514" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A514" s="30" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="515" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A515" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="516" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A516" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="517" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A517" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A518" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="519" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A519" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="520" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A520" s="30" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="521" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A521" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="522" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A522" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A523" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="524" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A524" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="525" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A525" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="526" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A526" s="30" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="527" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A527" s="30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="528" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A528" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="529" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A529" s="30" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="530" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A530" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="531" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A531" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="532" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A532" s="30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="533" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A533" s="30" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="534" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A534" s="30" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="535" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A535" s="30" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="536" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A536" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="537" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A537" s="30" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="538" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A538" s="30" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="539" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A539" s="30" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="540" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A540" s="30" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="541" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A541" s="30" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change Lookups sheet from veryHidden to hidden for easier inspection
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/QAReturns.xlsx
+++ b/output/QAReturns.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Lookups" state="veryHidden" r:id="rId4"/>
+    <sheet sheetId="1" name="Lookups" state="hidden" r:id="rId4"/>
     <sheet sheetId="2" name="Data Entry" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Tray Entry" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Product Returns" state="visible" r:id="rId7"/>
@@ -24501,7 +24501,7 @@
         <v>117</v>
       </c>
       <c r="B5" s="24">
-        <v>46083.13896923611</v>
+        <v>46083.139797916665</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -24517,7 +24517,7 @@
         <v>119</v>
       </c>
       <c r="B8" s="24">
-        <v>46083.13896923611</v>
+        <v>46083.139797916665</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix named ranges: switch from addEx to add method
addEx was silently failing to create named ranges. Using the
add(range, name) API correctly creates all 11 workbook-scoped
named ranges (Routes, Categories, Descriptions, Users, 5 route
area ranges, 2 category product ranges). Dropdowns now work.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/QAReturns.xlsx
+++ b/output/QAReturns.xlsx
@@ -13,6 +13,19 @@
     <sheet sheetId="7" name="Report Generator" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="VBA Code" state="visible" r:id="rId11"/>
   </sheets>
+  <definedNames>
+    <definedName name="Routes">Lookups!$A$2:$A$6</definedName>
+    <definedName name="Categories">Lookups!$B$2:$B$3</definedName>
+    <definedName name="Descriptions">Lookups!$C$2:$C$9</definedName>
+    <definedName name="Users">Lookups!$D$2:$D$5</definedName>
+    <definedName name="Route_City">Lookups!$E$2:$E$6</definedName>
+    <definedName name="Route_Out_of_Town">Lookups!$F$2:$F$18</definedName>
+    <definedName name="Route_Bacolod">Lookups!$G$2</definedName>
+    <definedName name="Route_Cebu">Lookups!$H$2</definedName>
+    <definedName name="Route_Davao">Lookups!$I$2</definedName>
+    <definedName name="Cat_Loaf">Lookups!$J$2:$J$10</definedName>
+    <definedName name="Cat_Assorted">Lookups!$K$2:$K$16</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -24501,7 +24514,7 @@
         <v>117</v>
       </c>
       <c r="B5" s="24">
-        <v>46083.139797916665</v>
+        <v>46083.14526261574</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -24517,7 +24530,7 @@
         <v>119</v>
       </c>
       <c r="B8" s="24">
-        <v>46083.139797916665</v>
+        <v>46083.14526261574</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Protect Created At column from manual editing
- Lock Created At cells (col P in Product Returns, col H in Tray Returns)
- Apply sheet protection with password on both data sheets
- VBA macros unprotect before writing and re-protect after
- Users can still edit all other columns normally

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/QAReturns.xlsx
+++ b/output/QAReturns.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="470">
   <si>
     <t>Routes</t>
   </si>
@@ -606,6 +606,9 @@
     <t xml:space="preserve">    ' ── Write data to Product Returns ──</t>
   </si>
   <si>
+    <t xml:space="preserve">    wsPR.Unprotect "qaReturns2026"</t>
+  </si>
+  <si>
     <t xml:space="preserve">    ' Col A (Record #) and Col B (Date Inspected) have formulas already</t>
   </si>
   <si>
@@ -654,6 +657,9 @@
     <t xml:space="preserve">    wsPR.Cells(nextRow, 16).NumberFormat = "DD MMM YYYY HH:MM"</t>
   </si>
   <si>
+    <t xml:space="preserve">    wsPR.Protect "qaReturns2026", True, True, True</t>
+  </si>
+  <si>
     <t xml:space="preserve">    ' ── Clear form ──</t>
   </si>
   <si>
@@ -750,6 +756,9 @@
     <t xml:space="preserve">    ' ── Write data to Tray Returns ──</t>
   </si>
   <si>
+    <t xml:space="preserve">    wsTR.Unprotect "qaReturns2026"</t>
+  </si>
+  <si>
     <t xml:space="preserve">    wsTR.Cells(nextRow, 3).Value = fRoute</t>
   </si>
   <si>
@@ -769,6 +778,9 @@
   </si>
   <si>
     <t xml:space="preserve">    wsTR.Cells(nextRow, 8).NumberFormat = "DD MMM YYYY HH:MM"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wsTR.Protect "qaReturns2026", True, True, True</t>
   </si>
   <si>
     <t xml:space="preserve">    wsForm.Range("A12").Value = "Record #" &amp; (nextRow - 1) &amp; " added successfully!"</t>
@@ -1604,18 +1616,28 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -13714,6 +13736,7 @@
       <c r="P501" s="16"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0" algorithmName="SHA-512" hashValue="1ssta8QaLaptHeH4QH1NMhNQucMCCM/r6JF8aJeelV3zgx/yI41RzoEbk0XxF6H6pDmGc+Fkow8iew3DvzhvdQ==" saltValue="JJcGS6w02klTUsDmoZM8JQ==" spinCount="100000"/>
   <conditionalFormatting sqref="J2:J501">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND(J2&lt;&gt;"",J2&lt;TODAY())</formula>
@@ -23796,6 +23819,7 @@
       <c r="H501" s="16"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0" algorithmName="SHA-512" hashValue="enjHApZnlEdXDw+V/LBgDXDrGbPBR+eMnVnZpVROrahG3vuFrGFmiJKuIUUP6DG/E93KDq1odE3NaJXdv2w7Ag==" saltValue="5A47lh4ZQ98H9dwljmvfKw==" spinCount="100000"/>
   <dataValidations count="506">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid" error="Please select from the list." sqref="C10:C501">
       <formula1>Routes</formula1>
@@ -25554,7 +25578,7 @@
         <v>118</v>
       </c>
       <c r="B5" s="26">
-        <v>46083.15656697917</v>
+        <v>46083.16065986111</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -25570,7 +25594,7 @@
         <v>120</v>
       </c>
       <c r="B8" s="26">
-        <v>46083.15656697917</v>
+        <v>46083.16065986111</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -25650,7 +25674,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A547"/>
+  <dimension ref="A1:A551"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="130" customWidth="1"/>
@@ -26158,17 +26182,17 @@
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="32" t="s">
-        <v>92</v>
+        <v>207</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="32" t="s">
-        <v>208</v>
+        <v>92</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
@@ -26233,17 +26257,17 @@
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="32" t="s">
-        <v>92</v>
+        <v>221</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="32" t="s">
-        <v>222</v>
+        <v>92</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
@@ -26253,27 +26277,27 @@
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="32" t="s">
-        <v>92</v>
+        <v>224</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="32" t="s">
-        <v>225</v>
+        <v>92</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="32" t="s">
-        <v>92</v>
+        <v>226</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="32" t="s">
-        <v>130</v>
+        <v>227</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
@@ -26283,62 +26307,62 @@
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="32" t="s">
-        <v>226</v>
+        <v>130</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="32" t="s">
-        <v>137</v>
+        <v>92</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="32" t="s">
-        <v>92</v>
+        <v>137</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="32" t="s">
-        <v>229</v>
+        <v>92</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="32" t="s">
-        <v>92</v>
+        <v>230</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="32" t="s">
-        <v>141</v>
+        <v>231</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" s="32" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" s="32" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" s="32" t="s">
-        <v>230</v>
+        <v>142</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="32" t="s">
-        <v>231</v>
+        <v>143</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
@@ -26348,217 +26372,217 @@
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" s="32" t="s">
-        <v>92</v>
+        <v>233</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="32" t="s">
-        <v>155</v>
+        <v>234</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" s="32" t="s">
-        <v>156</v>
+        <v>92</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" s="32" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" s="32" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" s="32" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="32" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="32" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" s="32" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" s="32" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="32" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" s="32" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="32" t="s">
-        <v>233</v>
+        <v>159</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" s="32" t="s">
-        <v>234</v>
+        <v>160</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="32" t="s">
-        <v>166</v>
+        <v>235</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" s="32" t="s">
-        <v>159</v>
+        <v>236</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" s="32" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" s="32" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="32" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="32" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="32" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" s="32" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="32" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" s="32" t="s">
-        <v>235</v>
+        <v>160</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="32" t="s">
-        <v>180</v>
+        <v>92</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" s="32" t="s">
-        <v>181</v>
+        <v>237</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" s="32" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" s="32" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" s="32" t="s">
-        <v>236</v>
+        <v>182</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" s="32" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" s="32" t="s">
-        <v>186</v>
+        <v>238</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" s="32" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" s="32" t="s">
-        <v>92</v>
+        <v>186</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" s="32" t="s">
-        <v>237</v>
+        <v>92</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" s="32" t="s">
-        <v>159</v>
+        <v>188</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" s="32" t="s">
-        <v>160</v>
+        <v>239</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" s="32" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" s="32" t="s">
-        <v>238</v>
+        <v>160</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" s="32" t="s">
-        <v>191</v>
+        <v>92</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" s="32" t="s">
-        <v>241</v>
+        <v>192</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.25">
@@ -26583,57 +26607,57 @@
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" s="32" t="s">
-        <v>92</v>
+        <v>246</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" s="32" t="s">
-        <v>207</v>
+        <v>247</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" s="32" t="s">
-        <v>208</v>
+        <v>248</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" s="32" t="s">
-        <v>209</v>
+        <v>249</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" s="32" t="s">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" s="32" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" s="32" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" s="32" t="s">
-        <v>92</v>
+        <v>211</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="32" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" s="32" t="s">
-        <v>246</v>
+        <v>213</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="32" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.25">
@@ -26643,82 +26667,82 @@
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" s="32" t="s">
-        <v>247</v>
+        <v>223</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" s="32" t="s">
-        <v>225</v>
+        <v>250</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" s="32" t="s">
-        <v>92</v>
+        <v>225</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A202" s="32" t="s">
-        <v>130</v>
+        <v>92</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" s="32" t="s">
-        <v>92</v>
+        <v>251</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" s="32" t="s">
-        <v>248</v>
+        <v>227</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" s="32" t="s">
-        <v>249</v>
+        <v>92</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" s="32" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" s="32" t="s">
-        <v>250</v>
+        <v>92</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" s="32" t="s">
-        <v>138</v>
+        <v>252</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A209" s="32" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A210" s="32" t="s">
-        <v>251</v>
+        <v>92</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A211" s="32" t="s">
-        <v>92</v>
+        <v>254</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A212" s="32" t="s">
-        <v>252</v>
+        <v>138</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A213" s="32" t="s">
-        <v>140</v>
+        <v>229</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A214" s="32" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.25">
@@ -26728,22 +26752,22 @@
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A216" s="32" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A217" s="32" t="s">
-        <v>254</v>
+        <v>140</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A218" s="32" t="s">
-        <v>255</v>
+        <v>231</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A219" s="32" t="s">
-        <v>256</v>
+        <v>92</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.25">
@@ -26753,87 +26777,87 @@
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A221" s="32" t="s">
-        <v>159</v>
+        <v>258</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A222" s="32" t="s">
-        <v>160</v>
+        <v>259</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A223" s="32" t="s">
-        <v>92</v>
+        <v>260</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A224" s="32" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A225" s="32" t="s">
-        <v>259</v>
+        <v>159</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A226" s="32" t="s">
-        <v>260</v>
+        <v>160</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A227" s="32" t="s">
-        <v>261</v>
+        <v>92</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A228" s="32" t="s">
-        <v>92</v>
+        <v>262</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A229" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A230" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A231" s="32" t="s">
-        <v>159</v>
+        <v>265</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A232" s="32" t="s">
-        <v>160</v>
+        <v>92</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A233" s="32" t="s">
-        <v>92</v>
+        <v>266</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A234" s="32" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A235" s="32" t="s">
-        <v>265</v>
+        <v>159</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A236" s="32" t="s">
-        <v>266</v>
+        <v>160</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A237" s="32" t="s">
-        <v>267</v>
+        <v>92</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.25">
@@ -26848,67 +26872,67 @@
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A240" s="32" t="s">
-        <v>92</v>
+        <v>270</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A241" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A242" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A243" s="32" t="s">
-        <v>92</v>
+        <v>273</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A244" s="32" t="s">
-        <v>272</v>
+        <v>92</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A245" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A246" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A247" s="32" t="s">
-        <v>275</v>
+        <v>92</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A248" s="32" t="s">
-        <v>182</v>
+        <v>276</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A249" s="32" t="s">
-        <v>183</v>
+        <v>277</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A250" s="32" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A251" s="32" t="s">
-        <v>187</v>
+        <v>279</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A252" s="32" t="s">
-        <v>277</v>
+        <v>182</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.25">
@@ -26918,7 +26942,7 @@
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A254" s="32" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.25">
@@ -26928,52 +26952,52 @@
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A256" s="32" t="s">
-        <v>92</v>
+        <v>281</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A257" s="32" t="s">
-        <v>279</v>
+        <v>183</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A258" s="32" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A259" s="32" t="s">
-        <v>281</v>
+        <v>187</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A260" s="32" t="s">
-        <v>282</v>
+        <v>92</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A261" s="32" t="s">
-        <v>92</v>
+        <v>283</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A262" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A263" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A264" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A265" s="32" t="s">
-        <v>286</v>
+        <v>92</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.25">
@@ -27008,37 +27032,37 @@
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A272" s="32" t="s">
-        <v>186</v>
+        <v>293</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A273" s="32" t="s">
-        <v>187</v>
+        <v>294</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A274" s="32" t="s">
-        <v>92</v>
+        <v>295</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A275" s="32" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A276" s="32" t="s">
-        <v>294</v>
+        <v>186</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A277" s="32" t="s">
-        <v>295</v>
+        <v>187</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A278" s="32" t="s">
-        <v>296</v>
+        <v>92</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.25">
@@ -27053,112 +27077,112 @@
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A281" s="32" t="s">
-        <v>159</v>
+        <v>299</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A282" s="32" t="s">
-        <v>160</v>
+        <v>300</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A283" s="32" t="s">
-        <v>92</v>
+        <v>301</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A284" s="32" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A285" s="32" t="s">
-        <v>300</v>
+        <v>159</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A286" s="32" t="s">
-        <v>301</v>
+        <v>160</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A287" s="32" t="s">
-        <v>284</v>
+        <v>92</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A288" s="32" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A289" s="32" t="s">
-        <v>287</v>
+        <v>304</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A290" s="32" t="s">
-        <v>288</v>
+        <v>305</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A291" s="32" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A292" s="32" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A293" s="32" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A294" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A295" s="32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A296" s="32" t="s">
-        <v>186</v>
+        <v>306</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A297" s="32" t="s">
-        <v>187</v>
+        <v>307</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A298" s="32" t="s">
-        <v>92</v>
+        <v>295</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A299" s="32" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A300" s="32" t="s">
-        <v>305</v>
+        <v>186</v>
       </c>
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A301" s="32" t="s">
-        <v>306</v>
+        <v>187</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A302" s="32" t="s">
-        <v>307</v>
+        <v>92</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.25">
@@ -27253,47 +27277,47 @@
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A321" s="32" t="s">
-        <v>291</v>
+        <v>326</v>
       </c>
     </row>
     <row r="322" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A322" s="32" t="s">
-        <v>292</v>
+        <v>327</v>
       </c>
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A323" s="32" t="s">
-        <v>186</v>
+        <v>328</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A324" s="32" t="s">
-        <v>187</v>
+        <v>329</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A325" s="32" t="s">
-        <v>92</v>
+        <v>295</v>
       </c>
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A326" s="32" t="s">
-        <v>326</v>
+        <v>296</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A327" s="32" t="s">
-        <v>327</v>
+        <v>186</v>
       </c>
     </row>
     <row r="328" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A328" s="32" t="s">
-        <v>328</v>
+        <v>187</v>
       </c>
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A329" s="32" t="s">
-        <v>329</v>
+        <v>92</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.25">
@@ -27318,27 +27342,27 @@
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A334" s="32" t="s">
-        <v>92</v>
+        <v>334</v>
       </c>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A335" s="32" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A336" s="32" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A337" s="32" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A338" s="32" t="s">
-        <v>337</v>
+        <v>92</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.25">
@@ -27373,42 +27397,42 @@
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A345" s="32" t="s">
-        <v>292</v>
+        <v>344</v>
       </c>
     </row>
     <row r="346" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A346" s="32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A347" s="32" t="s">
-        <v>187</v>
+        <v>346</v>
       </c>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A348" s="32" t="s">
-        <v>92</v>
+        <v>347</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A349" s="32" t="s">
-        <v>345</v>
+        <v>296</v>
       </c>
     </row>
     <row r="350" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A350" s="32" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="351" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A351" s="32" t="s">
-        <v>347</v>
+        <v>187</v>
       </c>
     </row>
     <row r="352" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A352" s="32" t="s">
-        <v>348</v>
+        <v>92</v>
       </c>
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.25">
@@ -27433,42 +27457,42 @@
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A357" s="32" t="s">
-        <v>92</v>
+        <v>353</v>
       </c>
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A358" s="32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A359" s="32" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A360" s="32" t="s">
-        <v>92</v>
+        <v>356</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A361" s="32" t="s">
-        <v>355</v>
+        <v>92</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A362" s="32" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A363" s="32" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A364" s="32" t="s">
-        <v>358</v>
+        <v>92</v>
       </c>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.25">
@@ -27478,27 +27502,27 @@
     </row>
     <row r="366" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A366" s="32" t="s">
-        <v>92</v>
+        <v>360</v>
       </c>
     </row>
     <row r="367" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A367" s="32" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A368" s="32" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A369" s="32" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="370" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A370" s="32" t="s">
-        <v>363</v>
+        <v>92</v>
       </c>
     </row>
     <row r="371" spans="1:1" x14ac:dyDescent="0.25">
@@ -27508,37 +27532,37 @@
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A372" s="32" t="s">
-        <v>92</v>
+        <v>365</v>
       </c>
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A373" s="32" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A374" s="32" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
     </row>
     <row r="375" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A375" s="32" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A376" s="32" t="s">
-        <v>363</v>
+        <v>92</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A377" s="32" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A378" s="32" t="s">
-        <v>92</v>
+        <v>365</v>
       </c>
     </row>
     <row r="379" spans="1:1" x14ac:dyDescent="0.25">
@@ -27558,7 +27582,7 @@
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A382" s="32" t="s">
-        <v>369</v>
+        <v>92</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.25">
@@ -27573,27 +27597,27 @@
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A385" s="32" t="s">
-        <v>92</v>
+        <v>372</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A386" s="32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="387" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A387" s="32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="388" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A388" s="32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="389" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A389" s="32" t="s">
-        <v>375</v>
+        <v>92</v>
       </c>
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.25">
@@ -27603,22 +27627,22 @@
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A391" s="32" t="s">
-        <v>92</v>
+        <v>377</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A392" s="32" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A393" s="32" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A394" s="32" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.25">
@@ -27628,17 +27652,17 @@
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A396" s="32" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="397" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A397" s="32" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="398" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A398" s="32" t="s">
-        <v>186</v>
+        <v>383</v>
       </c>
     </row>
     <row r="399" spans="1:1" x14ac:dyDescent="0.25">
@@ -27648,22 +27672,22 @@
     </row>
     <row r="400" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A400" s="32" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A401" s="32" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A402" s="32" t="s">
-        <v>384</v>
+        <v>186</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A403" s="32" t="s">
-        <v>385</v>
+        <v>92</v>
       </c>
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.25">
@@ -27678,27 +27702,27 @@
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A406" s="32" t="s">
-        <v>92</v>
+        <v>388</v>
       </c>
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A407" s="32" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A408" s="32" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A409" s="32" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A410" s="32" t="s">
-        <v>391</v>
+        <v>92</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.25">
@@ -27723,27 +27747,27 @@
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A415" s="32" t="s">
-        <v>292</v>
+        <v>396</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A416" s="32" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A417" s="32" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="418" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A418" s="32" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A419" s="32" t="s">
-        <v>399</v>
+        <v>296</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.25">
@@ -27773,47 +27797,47 @@
     </row>
     <row r="425" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A425" s="32" t="s">
-        <v>325</v>
+        <v>405</v>
       </c>
     </row>
     <row r="426" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A426" s="32" t="s">
-        <v>291</v>
+        <v>406</v>
       </c>
     </row>
     <row r="427" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A427" s="32" t="s">
-        <v>292</v>
+        <v>407</v>
       </c>
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A428" s="32" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A429" s="32" t="s">
-        <v>92</v>
+        <v>329</v>
       </c>
     </row>
     <row r="430" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A430" s="32" t="s">
-        <v>406</v>
+        <v>295</v>
       </c>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A431" s="32" t="s">
-        <v>407</v>
+        <v>296</v>
       </c>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A432" s="32" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A433" s="32" t="s">
-        <v>409</v>
+        <v>92</v>
       </c>
     </row>
     <row r="434" spans="1:1" x14ac:dyDescent="0.25">
@@ -27833,47 +27857,47 @@
     </row>
     <row r="437" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A437" s="32" t="s">
-        <v>92</v>
+        <v>413</v>
       </c>
     </row>
     <row r="438" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A438" s="32" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="439" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A439" s="32" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A440" s="32" t="s">
-        <v>386</v>
+        <v>416</v>
       </c>
     </row>
     <row r="441" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A441" s="32" t="s">
-        <v>385</v>
+        <v>92</v>
       </c>
     </row>
     <row r="442" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A442" s="32" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A443" s="32" t="s">
-        <v>92</v>
+        <v>418</v>
       </c>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A444" s="32" t="s">
-        <v>415</v>
+        <v>390</v>
       </c>
     </row>
     <row r="445" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A445" s="32" t="s">
-        <v>416</v>
+        <v>389</v>
       </c>
     </row>
     <row r="446" spans="1:1" x14ac:dyDescent="0.25">
@@ -27883,122 +27907,122 @@
     </row>
     <row r="447" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A447" s="32" t="s">
-        <v>392</v>
+        <v>92</v>
       </c>
     </row>
     <row r="448" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A448" s="32" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="449" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A449" s="32" t="s">
-        <v>292</v>
+        <v>420</v>
       </c>
     </row>
     <row r="450" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A450" s="32" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="451" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A451" s="32" t="s">
-        <v>92</v>
+        <v>396</v>
       </c>
     </row>
     <row r="452" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A452" s="32" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A453" s="32" t="s">
-        <v>383</v>
+        <v>296</v>
       </c>
     </row>
     <row r="454" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A454" s="32" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
     </row>
     <row r="455" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A455" s="32" t="s">
-        <v>386</v>
+        <v>92</v>
       </c>
     </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A456" s="32" t="s">
-        <v>385</v>
+        <v>422</v>
       </c>
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A457" s="32" t="s">
-        <v>419</v>
+        <v>387</v>
       </c>
     </row>
     <row r="458" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A458" s="32" t="s">
-        <v>92</v>
+        <v>418</v>
       </c>
     </row>
     <row r="459" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A459" s="32" t="s">
-        <v>420</v>
+        <v>390</v>
       </c>
     </row>
     <row r="460" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A460" s="32" t="s">
-        <v>421</v>
+        <v>389</v>
       </c>
     </row>
     <row r="461" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A461" s="32" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="462" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A462" s="32" t="s">
-        <v>423</v>
+        <v>92</v>
       </c>
     </row>
     <row r="463" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A463" s="32" t="s">
-        <v>391</v>
+        <v>424</v>
       </c>
     </row>
     <row r="464" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A464" s="32" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="465" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A465" s="32" t="s">
-        <v>396</v>
+        <v>426</v>
       </c>
     </row>
     <row r="466" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A466" s="32" t="s">
-        <v>92</v>
+        <v>427</v>
       </c>
     </row>
     <row r="467" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A467" s="32" t="s">
-        <v>425</v>
+        <v>395</v>
       </c>
     </row>
     <row r="468" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A468" s="32" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="469" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A469" s="32" t="s">
-        <v>427</v>
+        <v>400</v>
       </c>
     </row>
     <row r="470" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A470" s="32" t="s">
-        <v>428</v>
+        <v>92</v>
       </c>
     </row>
     <row r="471" spans="1:1" x14ac:dyDescent="0.25">
@@ -28023,37 +28047,37 @@
     </row>
     <row r="475" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A475" s="32" t="s">
-        <v>291</v>
+        <v>433</v>
       </c>
     </row>
     <row r="476" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A476" s="32" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="477" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A477" s="32" t="s">
-        <v>92</v>
+        <v>435</v>
       </c>
     </row>
     <row r="478" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A478" s="32" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="479" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A479" s="32" t="s">
-        <v>435</v>
+        <v>295</v>
       </c>
     </row>
     <row r="480" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A480" s="32" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="481" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A481" s="32" t="s">
-        <v>437</v>
+        <v>92</v>
       </c>
     </row>
     <row r="482" spans="1:1" x14ac:dyDescent="0.25">
@@ -28073,37 +28097,37 @@
     </row>
     <row r="485" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A485" s="32" t="s">
-        <v>325</v>
+        <v>441</v>
       </c>
     </row>
     <row r="486" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A486" s="32" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="487" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A487" s="32" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="488" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A488" s="32" t="s">
-        <v>92</v>
+        <v>444</v>
       </c>
     </row>
     <row r="489" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A489" s="32" t="s">
-        <v>443</v>
+        <v>329</v>
       </c>
     </row>
     <row r="490" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A490" s="32" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="491" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A491" s="32" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="492" spans="1:1" x14ac:dyDescent="0.25">
@@ -28113,22 +28137,22 @@
     </row>
     <row r="493" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A493" s="32" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="494" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A494" s="32" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="495" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A495" s="32" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="496" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A496" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="497" spans="1:1" x14ac:dyDescent="0.25">
@@ -28138,37 +28162,37 @@
     </row>
     <row r="498" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A498" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="499" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A499" s="32" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="500" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A500" s="32" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="501" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A501" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="502" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A502" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="503" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A503" s="32" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="504" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A504" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="505" spans="1:1" x14ac:dyDescent="0.25">
@@ -28178,212 +28202,232 @@
     </row>
     <row r="506" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A506" s="32" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="507" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A507" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="508" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A508" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="509" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A509" s="32" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
     </row>
     <row r="510" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A510" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="511" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A511" s="32" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="512" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A512" s="32" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="513" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A513" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="514" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A514" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="515" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A515" s="32" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
     </row>
     <row r="516" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A516" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="517" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A517" s="32" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="518" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A518" s="32" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="519" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A519" s="32" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="520" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A520" s="32" t="s">
-        <v>457</v>
+        <v>92</v>
       </c>
     </row>
     <row r="521" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A521" s="32" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
     </row>
     <row r="522" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A522" s="32" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
     </row>
     <row r="523" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A523" s="32" t="s">
-        <v>449</v>
+        <v>460</v>
       </c>
     </row>
     <row r="524" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A524" s="32" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
     </row>
     <row r="525" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A525" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="526" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A526" s="32" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="527" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A527" s="32" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="528" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A528" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="529" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A529" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="530" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A530" s="32" t="s">
-        <v>450</v>
+        <v>462</v>
       </c>
     </row>
     <row r="531" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A531" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="532" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A532" s="32" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
     </row>
     <row r="533" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A533" s="32" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="534" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A534" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="535" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A535" s="32" t="s">
-        <v>449</v>
+        <v>92</v>
       </c>
     </row>
     <row r="536" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A536" s="32" t="s">
-        <v>450</v>
+        <v>463</v>
       </c>
     </row>
     <row r="537" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A537" s="32" t="s">
-        <v>92</v>
+        <v>451</v>
       </c>
     </row>
     <row r="538" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A538" s="32" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="539" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A539" s="32" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
     </row>
     <row r="540" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A540" s="32" t="s">
-        <v>186</v>
+        <v>454</v>
       </c>
     </row>
     <row r="541" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A541" s="32" t="s">
-        <v>461</v>
+        <v>92</v>
       </c>
     </row>
     <row r="542" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A542" s="32" t="s">
-        <v>92</v>
+        <v>454</v>
       </c>
     </row>
     <row r="543" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A543" s="32" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="544" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A544" s="32" t="s">
-        <v>463</v>
+        <v>186</v>
       </c>
     </row>
     <row r="545" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A545" s="32" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="546" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A546" s="32" t="s">
-        <v>465</v>
+        <v>92</v>
       </c>
     </row>
     <row r="547" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A547" s="32" t="s">
-        <v>225</v>
+        <v>466</v>
+      </c>
+    </row>
+    <row r="548" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A548" s="32" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="549" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A549" s="32" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="550" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A550" s="32" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="551" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A551" s="32" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>